<commit_message>
fixed aggregate data fn
</commit_message>
<xml_diff>
--- a/data/EMP_DEETS.xlsx
+++ b/data/EMP_DEETS.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21267" windowHeight="8019"/>
+    <workbookView windowWidth="21267" windowHeight="8019" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="92">
   <si>
     <t>S. No.</t>
   </si>
@@ -285,6 +286,24 @@
   </si>
   <si>
     <t>NARAYAN RAO</t>
+  </si>
+  <si>
+    <t>SP NO</t>
+  </si>
+  <si>
+    <t>ALLOWED SHIFTS</t>
+  </si>
+  <si>
+    <t>IN-OT ALLOWED</t>
+  </si>
+  <si>
+    <t>OUT-OT ALLOWED</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>YES</t>
   </si>
 </sst>
 </file>
@@ -297,7 +316,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -309,21 +328,6 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="0"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -342,8 +346,16 @@
       <charset val="134"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -493,18 +505,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="42">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="1" tint="0.25"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -556,6 +562,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.25"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -700,12 +712,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -719,18 +725,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -747,6 +741,17 @@
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -761,30 +766,6 @@
       </top>
       <bottom style="thin">
         <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -849,6 +830,19 @@
         <color rgb="FF000000"/>
       </top>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -952,224 +946,237 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="9" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="9" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="12" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1500,651 +1507,651 @@
     <col min="6" max="6" width="16.1441441441441" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="28.8" spans="1:6">
-      <c r="A1" s="3" t="s">
+    <row r="1" s="26" customFormat="1" ht="28.8" spans="1:6">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="28" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="6">
+      <c r="A2" s="30">
         <v>1</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="8"/>
+      <c r="F2" s="4"/>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="6">
+      <c r="A3" s="30">
         <v>2</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="8"/>
+      <c r="F3" s="4"/>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="6">
+      <c r="A4" s="30">
         <v>3</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="8"/>
+      <c r="F4" s="4"/>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="6">
+      <c r="A5" s="30">
         <v>4</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="8"/>
+      <c r="F5" s="4"/>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="6">
+      <c r="A6" s="30">
         <v>5</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="8"/>
+      <c r="F6" s="4"/>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="6">
+      <c r="A7" s="30">
         <v>6</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="8"/>
+      <c r="F7" s="4"/>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="6">
+      <c r="A8" s="30">
         <v>7</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="6">
+      <c r="A9" s="30">
         <v>8</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="4" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="6">
+      <c r="A10" s="30">
         <v>9</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="12" t="s">
+      <c r="E10" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="F10" s="12" t="s">
+      <c r="F10" s="8" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="6">
+      <c r="A11" s="30">
         <v>10</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="6">
+      <c r="A12" s="30">
         <v>11</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="D12" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="6">
+      <c r="A13" s="30">
         <v>12</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="D13" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="6">
+      <c r="A14" s="30">
         <v>13</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="15" t="s">
+      <c r="C14" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="D14" s="16" t="s">
+      <c r="D14" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="E14" s="17" t="s">
+      <c r="E14" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="F14" s="17" t="s">
+      <c r="F14" s="12" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="6">
+      <c r="A15" s="30">
         <v>14</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="C15" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="D15" s="18" t="s">
+      <c r="D15" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="E15" s="17" t="s">
+      <c r="E15" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="F15" s="17" t="s">
+      <c r="F15" s="12" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="6">
+      <c r="A16" s="30">
         <v>15</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="C16" s="15" t="s">
+      <c r="C16" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="D16" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="E16" s="17" t="s">
+      <c r="E16" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="F16" s="17" t="s">
+      <c r="F16" s="12" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="6">
+      <c r="A17" s="30">
         <v>16</v>
       </c>
-      <c r="B17" s="14" t="s">
+      <c r="B17" s="33" t="s">
         <v>49</v>
       </c>
-      <c r="C17" s="15" t="s">
+      <c r="C17" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="D17" s="18" t="s">
+      <c r="D17" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="E17" s="17" t="s">
+      <c r="E17" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="F17" s="17" t="s">
+      <c r="F17" s="12" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="6">
+      <c r="A18" s="30">
         <v>17</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="C18" s="19" t="s">
+      <c r="C18" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="D18" s="18" t="s">
+      <c r="D18" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="E18" s="17" t="s">
+      <c r="E18" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="F18" s="17" t="s">
+      <c r="F18" s="12" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="6">
+      <c r="A19" s="30">
         <v>18</v>
       </c>
-      <c r="B19" s="20" t="s">
+      <c r="B19" s="34" t="s">
         <v>54</v>
       </c>
-      <c r="C19" s="21" t="s">
+      <c r="C19" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="D19" s="18" t="s">
+      <c r="D19" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="E19" s="22" t="s">
+      <c r="E19" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="F19" s="22" t="s">
+      <c r="F19" s="18" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="6">
+      <c r="A20" s="30">
         <v>19</v>
       </c>
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="C20" s="21" t="s">
+      <c r="C20" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="D20" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="E20" s="23" t="s">
+      <c r="E20" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="F20" s="22" t="s">
+      <c r="F20" s="18" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" s="6">
+      <c r="A21" s="30">
         <v>20</v>
       </c>
-      <c r="B21" s="20" t="s">
+      <c r="B21" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="C21" s="24" t="s">
+      <c r="C21" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="D21" s="25" t="s">
+      <c r="D21" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="E21" s="22" t="s">
+      <c r="E21" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="F21" s="22" t="s">
+      <c r="F21" s="18" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="6">
+      <c r="A22" s="30">
         <v>21</v>
       </c>
-      <c r="B22" s="20" t="s">
+      <c r="B22" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="C22" s="26" t="s">
+      <c r="C22" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="D22" s="27" t="s">
+      <c r="D22" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E22" s="22" t="s">
+      <c r="E22" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="F22" s="22" t="s">
+      <c r="F22" s="18" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="23" spans="1:6">
-      <c r="A23" s="6">
+      <c r="A23" s="30">
         <v>22</v>
       </c>
-      <c r="B23" s="20" t="s">
+      <c r="B23" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="C23" s="28" t="s">
+      <c r="C23" s="24" t="s">
         <v>64</v>
       </c>
-      <c r="D23" s="27" t="s">
+      <c r="D23" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E23" s="22" t="s">
+      <c r="E23" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="F23" s="22" t="s">
+      <c r="F23" s="18" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="6">
-        <v>23</v>
-      </c>
-      <c r="B24" s="20" t="s">
+      <c r="A24" s="30">
+        <v>23</v>
+      </c>
+      <c r="B24" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="C24" s="28" t="s">
+      <c r="C24" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="D24" s="27" t="s">
+      <c r="D24" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E24" s="22" t="s">
+      <c r="E24" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="F24" s="22" t="s">
+      <c r="F24" s="18" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="25" spans="1:6">
-      <c r="A25" s="6">
+      <c r="A25" s="30">
         <v>24</v>
       </c>
-      <c r="B25" s="20" t="s">
+      <c r="B25" s="34" t="s">
         <v>67</v>
       </c>
-      <c r="C25" s="29" t="s">
+      <c r="C25" s="25" t="s">
         <v>68</v>
       </c>
-      <c r="D25" s="27" t="s">
+      <c r="D25" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E25" s="22" t="s">
+      <c r="E25" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="F25" s="22" t="s">
+      <c r="F25" s="18" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="26" spans="1:6">
-      <c r="A26" s="6">
+      <c r="A26" s="30">
         <v>25</v>
       </c>
-      <c r="B26" s="20" t="s">
+      <c r="B26" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="C26" s="29" t="s">
+      <c r="C26" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="D26" s="27" t="s">
+      <c r="D26" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E26" s="22" t="s">
+      <c r="E26" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="F26" s="22" t="s">
+      <c r="F26" s="18" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27" s="6">
+      <c r="A27" s="30">
         <v>26</v>
       </c>
-      <c r="B27" s="20" t="s">
+      <c r="B27" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="C27" s="21" t="s">
+      <c r="C27" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="D27" s="27" t="s">
+      <c r="D27" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E27" s="22" t="s">
+      <c r="E27" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="F27" s="22" t="s">
+      <c r="F27" s="18" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="28" spans="1:6">
-      <c r="A28" s="6">
+      <c r="A28" s="30">
         <v>27</v>
       </c>
-      <c r="B28" s="20" t="s">
+      <c r="B28" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="C28" s="21" t="s">
+      <c r="C28" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="D28" s="27" t="s">
+      <c r="D28" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E28" s="22" t="s">
+      <c r="E28" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="F28" s="22" t="s">
+      <c r="F28" s="18" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="29" spans="1:6">
-      <c r="A29" s="6">
+      <c r="A29" s="30">
         <v>28</v>
       </c>
-      <c r="B29" s="20" t="s">
+      <c r="B29" s="34" t="s">
         <v>75</v>
       </c>
-      <c r="C29" s="28" t="s">
+      <c r="C29" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="D29" s="27" t="s">
+      <c r="D29" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E29" s="22" t="s">
+      <c r="E29" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="F29" s="22" t="s">
+      <c r="F29" s="18" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="30" spans="1:6">
-      <c r="A30" s="6">
+      <c r="A30" s="30">
         <v>29</v>
       </c>
-      <c r="B30" s="20" t="s">
+      <c r="B30" s="34" t="s">
         <v>77</v>
       </c>
-      <c r="C30" s="28" t="s">
+      <c r="C30" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="D30" s="27" t="s">
+      <c r="D30" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E30" s="22" t="s">
+      <c r="E30" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="F30" s="22" t="s">
+      <c r="F30" s="18" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="31" spans="1:6">
-      <c r="A31" s="6">
+      <c r="A31" s="30">
         <v>30</v>
       </c>
-      <c r="B31" s="20" t="s">
+      <c r="B31" s="34" t="s">
         <v>80</v>
       </c>
-      <c r="C31" s="28" t="s">
+      <c r="C31" s="24" t="s">
         <v>81</v>
       </c>
-      <c r="D31" s="27" t="s">
+      <c r="D31" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E31" s="22" t="s">
+      <c r="E31" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="F31" s="22" t="s">
+      <c r="F31" s="18" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="32" spans="1:6">
-      <c r="A32" s="6">
+      <c r="A32" s="30">
         <v>31</v>
       </c>
-      <c r="B32" s="20" t="s">
+      <c r="B32" s="34" t="s">
         <v>82</v>
       </c>
-      <c r="C32" s="24" t="s">
+      <c r="C32" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="D32" s="27" t="s">
+      <c r="D32" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E32" s="22" t="s">
+      <c r="E32" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="F32" s="22" t="s">
+      <c r="F32" s="18" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="33" spans="1:6">
-      <c r="A33" s="6">
+      <c r="A33" s="30">
         <v>32</v>
       </c>
-      <c r="B33" s="20" t="s">
+      <c r="B33" s="34" t="s">
         <v>84</v>
       </c>
-      <c r="C33" s="28" t="s">
+      <c r="C33" s="24" t="s">
         <v>85</v>
       </c>
-      <c r="D33" s="27" t="s">
+      <c r="D33" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E33" s="22" t="s">
+      <c r="E33" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="F33" s="22" t="s">
+      <c r="F33" s="18" t="s">
         <v>48</v>
       </c>
     </row>
@@ -2152,4 +2159,772 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:G33"/>
+  <sheetFormatPr defaultColWidth="8.79279279279279" defaultRowHeight="14.4" outlineLevelCol="6"/>
+  <cols>
+    <col min="1" max="1" width="15.1801801801802" customWidth="1"/>
+    <col min="2" max="2" width="24.7387387387387" customWidth="1"/>
+    <col min="3" max="3" width="20.8738738738739" customWidth="1"/>
+    <col min="4" max="4" width="5.69369369369369" customWidth="1"/>
+    <col min="5" max="5" width="16.5675675675676" customWidth="1"/>
+    <col min="6" max="6" width="15.7567567567568" customWidth="1"/>
+    <col min="7" max="7" width="17.954954954955" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="1" customFormat="1" spans="1:7">
+      <c r="A1" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="4"/>
+      <c r="F2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="4"/>
+      <c r="F3" t="s">
+        <v>90</v>
+      </c>
+      <c r="G3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4" t="s">
+        <v>90</v>
+      </c>
+      <c r="G4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5" t="s">
+        <v>90</v>
+      </c>
+      <c r="G5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="F6" t="s">
+        <v>90</v>
+      </c>
+      <c r="G6" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="4"/>
+      <c r="F7" t="s">
+        <v>90</v>
+      </c>
+      <c r="G7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" t="s">
+        <v>90</v>
+      </c>
+      <c r="G8" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" t="s">
+        <v>90</v>
+      </c>
+      <c r="G9" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" t="s">
+        <v>90</v>
+      </c>
+      <c r="G10" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11" t="s">
+        <v>90</v>
+      </c>
+      <c r="G11" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" t="s">
+        <v>90</v>
+      </c>
+      <c r="G12" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13" t="s">
+        <v>90</v>
+      </c>
+      <c r="G13" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F14" t="s">
+        <v>90</v>
+      </c>
+      <c r="G14" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" t="s">
+        <v>90</v>
+      </c>
+      <c r="G15" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="F16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G16" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F17" t="s">
+        <v>90</v>
+      </c>
+      <c r="G17" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F18" t="s">
+        <v>90</v>
+      </c>
+      <c r="G18" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="E19" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="F19" t="s">
+        <v>90</v>
+      </c>
+      <c r="G19" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="C20" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="E20" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="F20" t="s">
+        <v>90</v>
+      </c>
+      <c r="G20" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="B21" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="C21" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="D21" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="E21" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="F21" t="s">
+        <v>90</v>
+      </c>
+      <c r="G21" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="B22" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="D22" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="E22" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="F22" t="s">
+        <v>90</v>
+      </c>
+      <c r="G22" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="B23" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="D23" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="E23" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="F23" t="s">
+        <v>90</v>
+      </c>
+      <c r="G23" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="B24" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="C24" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="D24" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="E24" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="F24" t="s">
+        <v>90</v>
+      </c>
+      <c r="G24" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="B25" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="D25" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="E25" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="F25" t="s">
+        <v>90</v>
+      </c>
+      <c r="G25" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="B26" s="25" t="s">
+        <v>70</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="D26" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="E26" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="F26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G26" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="B27" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="C27" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="D27" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="E27" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="F27" t="s">
+        <v>90</v>
+      </c>
+      <c r="G27" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="B28" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="C28" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="D28" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="E28" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="F28" t="s">
+        <v>90</v>
+      </c>
+      <c r="G28" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="B29" s="24" t="s">
+        <v>76</v>
+      </c>
+      <c r="C29" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="E29" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="F29" t="s">
+        <v>90</v>
+      </c>
+      <c r="G29" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="B30" s="24" t="s">
+        <v>78</v>
+      </c>
+      <c r="C30" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="D30" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="E30" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="F30" t="s">
+        <v>90</v>
+      </c>
+      <c r="G30" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="B31" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="C31" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="D31" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="E31" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="F31" t="s">
+        <v>90</v>
+      </c>
+      <c r="G31" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="B32" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="C32" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="D32" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="E32" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="F32" t="s">
+        <v>90</v>
+      </c>
+      <c r="G32" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="B33" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="C33" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="D33" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="E33" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="F33" t="s">
+        <v>90</v>
+      </c>
+      <c r="G33" t="s">
+        <v>91</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>